<commit_message>
Modified schema (removed check constraint from Question model
</commit_message>
<xml_diff>
--- a/docs/2schema.xlsx
+++ b/docs/2schema.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Farheen\TestSeries\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04F1EB8B-E724-4203-B21F-0D0ECDFAC187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4822649-6CA8-4DD0-B155-EC23B81BFA3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13224" yWindow="3192" windowWidth="8952" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="152">
   <si>
     <t>Field</t>
   </si>
@@ -463,9 +463,6 @@
   </si>
   <si>
     <t>Plain text extracted from the answer content</t>
-  </si>
-  <si>
-    <t>CHECK (question_type IN ('THEORY', 'MCQ', 'CASE_STUDY', 'TABLE', 'HYBRID'))</t>
   </si>
   <si>
     <t>Paper type (RTP, PYQ or MOCK)</t>
@@ -859,7 +856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D152"/>
+  <dimension ref="A1:D149"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:4" ht="23.4">
@@ -1565,413 +1562,403 @@
         <v>80</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="18">
-      <c r="A77" s="5" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4">
-      <c r="A79" s="4" t="s">
+    <row r="78" spans="1:4" ht="18">
+      <c r="A78" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="23.4">
+      <c r="A84" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="28.8">
+      <c r="A86" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="57.6">
+      <c r="A87" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="72">
+      <c r="A88" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="86.4">
+      <c r="A89" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="86.4">
+      <c r="A90" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="57.6">
+      <c r="A91" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D91" s="2" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="18">
-      <c r="A81" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4">
-      <c r="A83" s="4" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" ht="23.4">
-      <c r="A87" s="3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" ht="28.8">
-      <c r="A89" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D89" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" ht="57.6">
-      <c r="A90" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="72">
-      <c r="A91" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B91" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" ht="86.4">
+    <row r="92" spans="1:4" ht="72">
       <c r="A92" s="2" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>127</v>
+        <v>9</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" ht="86.4">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="72">
       <c r="A93" s="2" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="B93" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="18">
+      <c r="A95" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
+      <c r="A97" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="23.4">
+      <c r="A101" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" ht="28.8">
+      <c r="A103" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" ht="57.6">
+      <c r="A104" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" ht="100.8">
+      <c r="A105" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B105" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C93" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" ht="57.6">
-      <c r="A94" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B94" s="2" t="s">
+      <c r="C105" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" ht="86.4">
+      <c r="A106" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" ht="100.8">
+      <c r="A107" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="18">
+      <c r="A109" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4">
+      <c r="A111" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="23.4">
+      <c r="A115" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" ht="28.8">
+      <c r="A117" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" ht="57.6">
+      <c r="A118" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" ht="86.4">
+      <c r="A119" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" ht="28.8">
+      <c r="A120" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B120" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="C120" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D94" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" ht="72">
-      <c r="A95" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B95" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="72">
-      <c r="A96" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" ht="18">
-      <c r="A98" s="5" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4">
-      <c r="A100" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" ht="23.4">
-      <c r="A104" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" ht="28.8">
-      <c r="A106" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B106" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C106" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D106" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" ht="57.6">
-      <c r="A107" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" ht="100.8">
-      <c r="A108" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B108" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C108" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="D108" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" ht="86.4">
-      <c r="A109" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B109" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C109" s="2" t="s">
+      <c r="D120" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" ht="100.8">
-      <c r="A110" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B110" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" ht="18">
-      <c r="A112" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4">
-      <c r="A114" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" ht="23.4">
-      <c r="A118" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" ht="28.8">
-      <c r="A120" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B120" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D120" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="121" spans="1:4" ht="57.6">
       <c r="A121" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" ht="86.4">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" ht="57.6">
       <c r="A122" s="2" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>138</v>
+        <v>64</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" ht="28.8">
-      <c r="A123" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B123" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C123" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D123" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" ht="31.2">
+      <c r="A125" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" ht="18">
+      <c r="A127" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4">
+      <c r="A128" s="6"/>
+    </row>
+    <row r="129" spans="1:1">
+      <c r="A129" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130" s="6"/>
+    </row>
+    <row r="131" spans="1:1">
+      <c r="A131" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132" s="6"/>
+    </row>
+    <row r="133" spans="1:1">
+      <c r="A133" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1">
+      <c r="A134" s="6"/>
+    </row>
+    <row r="135" spans="1:1">
+      <c r="A135" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" ht="18">
+      <c r="A137" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1">
+      <c r="A138" s="6"/>
+    </row>
+    <row r="139" spans="1:1">
+      <c r="A139" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1">
+      <c r="A140" s="6"/>
+    </row>
+    <row r="141" spans="1:1">
+      <c r="A141" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" ht="18">
+      <c r="A143" s="5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1">
+      <c r="A144" s="6"/>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145" s="6" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="57.6">
-      <c r="A124" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" ht="57.6">
-      <c r="A125" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B125" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C125" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D125" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" ht="31.2">
-      <c r="A128" s="7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="130" spans="1:1" ht="18">
-      <c r="A130" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="131" spans="1:1">
-      <c r="A131" s="6"/>
-    </row>
-    <row r="132" spans="1:1">
-      <c r="A132" s="6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="133" spans="1:1">
-      <c r="A133" s="6"/>
-    </row>
-    <row r="134" spans="1:1">
-      <c r="A134" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="135" spans="1:1">
-      <c r="A135" s="6"/>
-    </row>
-    <row r="136" spans="1:1">
-      <c r="A136" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="137" spans="1:1">
-      <c r="A137" s="6"/>
-    </row>
-    <row r="138" spans="1:1">
-      <c r="A138" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="140" spans="1:1" ht="18">
-      <c r="A140" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="141" spans="1:1">
-      <c r="A141" s="6"/>
-    </row>
-    <row r="142" spans="1:1">
-      <c r="A142" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="143" spans="1:1">
-      <c r="A143" s="6"/>
-    </row>
-    <row r="144" spans="1:1">
-      <c r="A144" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="146" spans="1:1" ht="18">
-      <c r="A146" s="5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="147" spans="1:1">
-      <c r="A147" s="6"/>
+    <row r="147" spans="1:1" ht="18">
+      <c r="A147" s="5" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="148" spans="1:1">
-      <c r="A148" s="6" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="150" spans="1:1" ht="18">
-      <c r="A150" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="151" spans="1:1">
-      <c r="A151" s="6"/>
-    </row>
-    <row r="152" spans="1:1">
-      <c r="A152" s="6" t="s">
+      <c r="A148" s="6"/>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149" s="6" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Modified schema (added chapter_keyword model), implementing phase 3c automatic chapter mapping
</commit_message>
<xml_diff>
--- a/docs/2schema.xlsx
+++ b/docs/2schema.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Farheen\TestSeries\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4822649-6CA8-4DD0-B155-EC23B81BFA3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B70246EA-0909-4DF2-8205-689807140D98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13224" yWindow="3192" windowWidth="8952" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="164">
   <si>
     <t>Field</t>
   </si>
@@ -481,6 +481,42 @@
   </si>
   <si>
     <t>idx_generated_paper_user</t>
+  </si>
+  <si>
+    <t>Constraint</t>
+  </si>
+  <si>
+    <t>chapter_keyword_id</t>
+  </si>
+  <si>
+    <t>BIGINT</t>
+  </si>
+  <si>
+    <t>PK, NOT NULL</t>
+  </si>
+  <si>
+    <t>keywords</t>
+  </si>
+  <si>
+    <t>Chapter Keyword</t>
+  </si>
+  <si>
+    <t>Unique keyword record identifier</t>
+  </si>
+  <si>
+    <t>FK → Chapter(chapter_id), NOT NULL, ON DELETE CASCADE</t>
+  </si>
+  <si>
+    <t>Associated chapter</t>
+  </si>
+  <si>
+    <t>Normalized keywords, one keyword per line, used by the deterministic chapter mapping engine</t>
+  </si>
+  <si>
+    <t>Additional Constraints</t>
+  </si>
+  <si>
+    <t>UNIQUE(chapter_id)</t>
   </si>
 </sst>
 </file>
@@ -553,7 +589,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -574,6 +610,9 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -856,7 +895,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D149"/>
+  <dimension ref="A1:D163"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:4" ht="23.4">
@@ -1873,85 +1912,141 @@
         <v>120</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="31.2">
-      <c r="A125" s="7" t="s">
+    <row r="125" spans="1:4" ht="43.2" customHeight="1">
+      <c r="A125" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" ht="28.8">
+      <c r="A127" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" ht="57.6">
+      <c r="A128" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" ht="115.2">
+      <c r="A129" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" ht="187.2">
+      <c r="A130" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" ht="57.6">
+      <c r="A131" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" ht="57.6">
+      <c r="A132" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" ht="14.4" customHeight="1"/>
+    <row r="134" spans="1:4" ht="28.8" customHeight="1">
+      <c r="A134" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" ht="40.200000000000003" customHeight="1">
+      <c r="A135" s="8"/>
+    </row>
+    <row r="136" spans="1:4" ht="27" customHeight="1">
+      <c r="A136" s="4" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" ht="31.2">
+      <c r="A139" s="7" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="127" spans="1:4" ht="18">
-      <c r="A127" s="5" t="s">
+    <row r="141" spans="1:4" ht="18">
+      <c r="A141" s="5" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="128" spans="1:4">
-      <c r="A128" s="6"/>
-    </row>
-    <row r="129" spans="1:1">
-      <c r="A129" s="6" t="s">
+    <row r="142" spans="1:4">
+      <c r="A142" s="6"/>
+    </row>
+    <row r="143" spans="1:4">
+      <c r="A143" s="6" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="130" spans="1:1">
-      <c r="A130" s="6"/>
-    </row>
-    <row r="131" spans="1:1">
-      <c r="A131" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="132" spans="1:1">
-      <c r="A132" s="6"/>
-    </row>
-    <row r="133" spans="1:1">
-      <c r="A133" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="134" spans="1:1">
-      <c r="A134" s="6"/>
-    </row>
-    <row r="135" spans="1:1">
-      <c r="A135" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="137" spans="1:1" ht="18">
-      <c r="A137" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="138" spans="1:1">
-      <c r="A138" s="6"/>
-    </row>
-    <row r="139" spans="1:1">
-      <c r="A139" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="140" spans="1:1">
-      <c r="A140" s="6"/>
-    </row>
-    <row r="141" spans="1:1">
-      <c r="A141" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="143" spans="1:1" ht="18">
-      <c r="A143" s="5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="144" spans="1:1">
+    <row r="144" spans="1:4">
       <c r="A144" s="6"/>
     </row>
     <row r="145" spans="1:1">
       <c r="A145" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="147" spans="1:1" ht="18">
-      <c r="A147" s="5" t="s">
-        <v>43</v>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1">
+      <c r="A146" s="6"/>
+    </row>
+    <row r="147" spans="1:1">
+      <c r="A147" s="6" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="148" spans="1:1">
@@ -1959,6 +2054,53 @@
     </row>
     <row r="149" spans="1:1">
       <c r="A149" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" ht="18">
+      <c r="A151" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152" s="6"/>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1">
+      <c r="A154" s="6"/>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" ht="18">
+      <c r="A157" s="5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1">
+      <c r="A158" s="6"/>
+    </row>
+    <row r="159" spans="1:1">
+      <c r="A159" s="6" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" ht="18">
+      <c r="A161" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1">
+      <c r="A162" s="6"/>
+    </row>
+    <row r="163" spans="1:1">
+      <c r="A163" s="6" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated schema, added instruction type in question model
</commit_message>
<xml_diff>
--- a/docs/2schema.xlsx
+++ b/docs/2schema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Farheen\TestSeries\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B70246EA-0909-4DF2-8205-689807140D98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2F7578-7124-4E67-AE48-27AE32793FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -171,9 +171,6 @@
     <t>question_type</t>
   </si>
   <si>
-    <t>marks</t>
-  </si>
-  <si>
     <t>source_page</t>
   </si>
   <si>
@@ -336,12 +333,6 @@
     <t>Sub-question identifier (e.g., a, b, i, ii)</t>
   </si>
   <si>
-    <t>Type of question</t>
-  </si>
-  <si>
-    <t>Marks allocated to the question</t>
-  </si>
-  <si>
     <t>Page number in the source PDF</t>
   </si>
   <si>
@@ -517,6 +508,15 @@
   </si>
   <si>
     <t>UNIQUE(chapter_id)</t>
+  </si>
+  <si>
+    <t>instruction_type</t>
+  </si>
+  <si>
+    <t>Primary instruction verb detected from the question (e.g., EXPLAIN, DEFINE, CALCULATE, PREPARE, DISCUSS).</t>
+  </si>
+  <si>
+    <t>Type of question (High level question type)</t>
   </si>
 </sst>
 </file>
@@ -900,7 +900,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="23.4">
       <c r="A1" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28.8">
@@ -928,7 +928,7 @@
         <v>5</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="28.8">
@@ -942,7 +942,7 @@
         <v>9</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="43.2">
@@ -995,10 +995,10 @@
         <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="57.6">
@@ -1009,7 +1009,7 @@
         <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>23</v>
@@ -1017,7 +1017,7 @@
     </row>
     <row r="13" spans="1:4" ht="23.4">
       <c r="A13" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="28.8">
@@ -1045,7 +1045,7 @@
         <v>5</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="43.2">
@@ -1073,7 +1073,7 @@
         <v>9</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="72">
@@ -1087,7 +1087,7 @@
         <v>18</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="57.6">
@@ -1098,15 +1098,15 @@
         <v>21</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="23.4">
       <c r="A23" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="28.8">
@@ -1134,7 +1134,7 @@
         <v>5</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="86.4">
@@ -1145,15 +1145,15 @@
         <v>36</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="57.6">
       <c r="A28" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>8</v>
@@ -1162,12 +1162,12 @@
         <v>9</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="57.6">
       <c r="A29" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>36</v>
@@ -1176,7 +1176,7 @@
         <v>37</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="57.6">
@@ -1187,25 +1187,25 @@
         <v>21</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="18">
       <c r="A32" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="23.4">
       <c r="A38" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="46.8" customHeight="1">
@@ -1233,7 +1233,7 @@
         <v>5</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="72">
@@ -1244,10 +1244,10 @@
         <v>36</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4">
@@ -1258,7 +1258,7 @@
         <v>36</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>30</v>
@@ -1275,7 +1275,7 @@
         <v>9</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="72">
@@ -1289,12 +1289,12 @@
         <v>9</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="57.6">
       <c r="A46" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>36</v>
@@ -1303,12 +1303,12 @@
         <v>9</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="100.8">
       <c r="A47" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>33</v>
@@ -1317,12 +1317,12 @@
         <v>37</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="72">
       <c r="A48" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>34</v>
@@ -1331,7 +1331,7 @@
         <v>9</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="43.2">
@@ -1345,7 +1345,7 @@
         <v>37</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="28.8">
@@ -1359,7 +1359,7 @@
         <v>9</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="57.6">
@@ -1370,25 +1370,25 @@
         <v>21</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="18">
       <c r="A53" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="23.4">
       <c r="A59" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="28.8">
@@ -1407,7 +1407,7 @@
     </row>
     <row r="62" spans="1:4" ht="57.6">
       <c r="A62" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>4</v>
@@ -1416,21 +1416,21 @@
         <v>5</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="129.6">
       <c r="A63" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4">
@@ -1441,7 +1441,7 @@
         <v>36</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>41</v>
@@ -1455,10 +1455,10 @@
         <v>36</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="86.4">
@@ -1472,26 +1472,26 @@
         <v>9</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="72">
       <c r="A67" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72">
       <c r="A68" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>34</v>
@@ -1500,7 +1500,7 @@
         <v>9</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="72">
@@ -1514,12 +1514,12 @@
         <v>9</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="72">
       <c r="A70" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>34</v>
@@ -1528,7 +1528,7 @@
         <v>9</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="72">
@@ -1542,10 +1542,10 @@
         <v>9</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="28.8">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="60" customHeight="1">
       <c r="A72" s="2" t="s">
         <v>47</v>
       </c>
@@ -1556,26 +1556,26 @@
         <v>9</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" ht="57.6">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="201.6">
       <c r="A73" s="2" t="s">
-        <v>48</v>
+        <v>161</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>104</v>
+        <v>162</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="72">
       <c r="A74" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>36</v>
@@ -1584,7 +1584,7 @@
         <v>37</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="57.6">
@@ -1595,25 +1595,25 @@
         <v>21</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="18">
       <c r="A78" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="23.4">
       <c r="A84" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="28.8">
@@ -1632,7 +1632,7 @@
     </row>
     <row r="87" spans="1:4" ht="57.6">
       <c r="A87" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>4</v>
@@ -1641,7 +1641,7 @@
         <v>5</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="72">
@@ -1652,10 +1652,10 @@
         <v>36</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="89" spans="1:4" ht="86.4">
@@ -1666,10 +1666,10 @@
         <v>36</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="86.4">
@@ -1680,15 +1680,15 @@
         <v>36</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="57.6">
       <c r="A91" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>33</v>
@@ -1697,12 +1697,12 @@
         <v>9</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="72">
       <c r="A92" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>36</v>
@@ -1711,36 +1711,36 @@
         <v>9</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="72">
       <c r="A93" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="18">
       <c r="A95" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="101" spans="1:4" ht="23.4">
       <c r="A101" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="28.8">
@@ -1759,7 +1759,7 @@
     </row>
     <row r="104" spans="1:4" ht="57.6">
       <c r="A104" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>4</v>
@@ -1768,40 +1768,40 @@
         <v>5</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="105" spans="1:4" ht="100.8">
       <c r="A105" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="106" spans="1:4" ht="86.4">
       <c r="A106" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="107" spans="1:4" ht="100.8">
       <c r="A107" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>36</v>
@@ -1810,22 +1810,22 @@
         <v>9</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="109" spans="1:4" ht="18">
       <c r="A109" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="115" spans="1:4" ht="23.4">
       <c r="A115" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="28.8">
@@ -1844,7 +1844,7 @@
     </row>
     <row r="118" spans="1:4" ht="57.6">
       <c r="A118" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>4</v>
@@ -1853,7 +1853,7 @@
         <v>5</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="119" spans="1:4" ht="86.4">
@@ -1864,7 +1864,7 @@
         <v>36</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D119" s="2" t="s">
         <v>41</v>
@@ -1872,7 +1872,7 @@
     </row>
     <row r="120" spans="1:4" ht="28.8">
       <c r="A120" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>33</v>
@@ -1881,12 +1881,12 @@
         <v>9</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="121" spans="1:4" ht="57.6">
       <c r="A121" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>34</v>
@@ -1895,7 +1895,7 @@
         <v>37</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="122" spans="1:4" ht="57.6">
@@ -1906,15 +1906,15 @@
         <v>21</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="125" spans="1:4" ht="43.2" customHeight="1">
       <c r="A125" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="127" spans="1:4" ht="28.8">
@@ -1925,7 +1925,7 @@
         <v>1</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D127" s="1" t="s">
         <v>2</v>
@@ -1933,16 +1933,16 @@
     </row>
     <row r="128" spans="1:4" ht="57.6">
       <c r="A128" s="2" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C128" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D128" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="D128" s="2" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="129" spans="1:4" ht="115.2">
@@ -1953,15 +1953,15 @@
         <v>36</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="130" spans="1:4" ht="187.2">
       <c r="A130" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>34</v>
@@ -1970,7 +1970,7 @@
         <v>9</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="131" spans="1:4" ht="57.6">
@@ -1981,10 +1981,10 @@
         <v>21</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="132" spans="1:4" ht="57.6">
@@ -1995,7 +1995,7 @@
         <v>21</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D132" s="2" t="s">
         <v>23</v>
@@ -2004,7 +2004,7 @@
     <row r="133" spans="1:4" ht="14.4" customHeight="1"/>
     <row r="134" spans="1:4" ht="28.8" customHeight="1">
       <c r="A134" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="135" spans="1:4" ht="40.200000000000003" customHeight="1">
@@ -2012,17 +2012,17 @@
     </row>
     <row r="136" spans="1:4" ht="27" customHeight="1">
       <c r="A136" s="4" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="139" spans="1:4" ht="31.2">
       <c r="A139" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="141" spans="1:4" ht="18">
       <c r="A141" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -2030,7 +2030,7 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -2038,7 +2038,7 @@
     </row>
     <row r="145" spans="1:1">
       <c r="A145" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="146" spans="1:1">
@@ -2046,7 +2046,7 @@
     </row>
     <row r="147" spans="1:1">
       <c r="A147" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="148" spans="1:1">
@@ -2054,12 +2054,12 @@
     </row>
     <row r="149" spans="1:1">
       <c r="A149" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="151" spans="1:1" ht="18">
       <c r="A151" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="152" spans="1:1">
@@ -2067,7 +2067,7 @@
     </row>
     <row r="153" spans="1:1">
       <c r="A153" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="154" spans="1:1">
@@ -2075,12 +2075,12 @@
     </row>
     <row r="155" spans="1:1">
       <c r="A155" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="157" spans="1:1" ht="18">
       <c r="A157" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="158" spans="1:1">
@@ -2088,7 +2088,7 @@
     </row>
     <row r="159" spans="1:1">
       <c r="A159" s="6" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="161" spans="1:1" ht="18">
@@ -2101,7 +2101,7 @@
     </row>
     <row r="163" spans="1:1">
       <c r="A163" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated schema, added marks, index and check constraint
</commit_message>
<xml_diff>
--- a/docs/2schema.xlsx
+++ b/docs/2schema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Farheen\TestSeries\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2F7578-7124-4E67-AE48-27AE32793FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E7E1593-F61A-4BD4-9CDD-C4313C886DA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="170">
   <si>
     <t>Field</t>
   </si>
@@ -171,6 +171,9 @@
     <t>question_type</t>
   </si>
   <si>
+    <t>marks</t>
+  </si>
+  <si>
     <t>source_page</t>
   </si>
   <si>
@@ -513,10 +516,50 @@
     <t>instruction_type</t>
   </si>
   <si>
-    <t>Primary instruction verb detected from the question (e.g., EXPLAIN, DEFINE, CALCULATE, PREPARE, DISCUSS).</t>
-  </si>
-  <si>
-    <t>Type of question (High level question type)</t>
+    <t>Marks allocated to the question, if detected from the document.</t>
+  </si>
+  <si>
+    <t>High-level category of the question
+(THEORY, PRACTICAL, CASE_STUDY, OBJECTIVE, MIXED, UNIDENTIFIED)</t>
+  </si>
+  <si>
+    <t>Primary instruction verb extracted from the question
+(e.g., DEFINE, EXPLAIN, DISCUSS, PREPARE, CALCULATE, ANALYSE)</t>
+  </si>
+  <si>
+    <t>CHECK CONSRAINT</t>
+  </si>
+  <si>
+    <t>CHECK (
+question_type IN (
+'THEORY',
+'PRACTICAL',
+'CASE_STUDY',
+'OBJECTIVE',
+'MIXED',
+'UNIDENTIFIED'
+))</t>
+  </si>
+  <si>
+    <t>CHECK (
+instruction_type IN (
+'DEFINE',
+'EXPLAIN',
+'DISCUSS',
+'STATE',
+'LIST',
+'COMPARE',
+'DIFFERENTIATE',
+'CALCULATE',
+'COMPUTE',
+'PREPARE',
+'JOURNALIZE',
+'ANALYSE',
+'DETERMINE'
+))</t>
+  </si>
+  <si>
+    <t>idx_question_instruction_type</t>
   </si>
 </sst>
 </file>
@@ -589,7 +632,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -614,6 +657,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -895,12 +942,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D163"/>
+  <dimension ref="A1:D171"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:4" ht="23.4">
       <c r="A1" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28.8">
@@ -928,7 +975,7 @@
         <v>5</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="28.8">
@@ -942,7 +989,7 @@
         <v>9</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="43.2">
@@ -995,10 +1042,10 @@
         <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="57.6">
@@ -1009,7 +1056,7 @@
         <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>23</v>
@@ -1017,7 +1064,7 @@
     </row>
     <row r="13" spans="1:4" ht="23.4">
       <c r="A13" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="28.8">
@@ -1045,7 +1092,7 @@
         <v>5</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="43.2">
@@ -1073,7 +1120,7 @@
         <v>9</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="72">
@@ -1087,7 +1134,7 @@
         <v>18</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="57.6">
@@ -1098,15 +1145,15 @@
         <v>21</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="23.4">
       <c r="A23" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="28.8">
@@ -1134,7 +1181,7 @@
         <v>5</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="86.4">
@@ -1145,15 +1192,15 @@
         <v>36</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="57.6">
       <c r="A28" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>8</v>
@@ -1162,12 +1209,12 @@
         <v>9</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="57.6">
       <c r="A29" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>36</v>
@@ -1176,7 +1223,7 @@
         <v>37</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="57.6">
@@ -1187,25 +1234,25 @@
         <v>21</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="18">
       <c r="A32" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="23.4">
       <c r="A38" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="46.8" customHeight="1">
@@ -1233,7 +1280,7 @@
         <v>5</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="72">
@@ -1244,10 +1291,10 @@
         <v>36</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4">
@@ -1258,7 +1305,7 @@
         <v>36</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>30</v>
@@ -1275,7 +1322,7 @@
         <v>9</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="72">
@@ -1289,12 +1336,12 @@
         <v>9</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="57.6">
       <c r="A46" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>36</v>
@@ -1303,12 +1350,12 @@
         <v>9</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="100.8">
       <c r="A47" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>33</v>
@@ -1317,12 +1364,12 @@
         <v>37</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="72">
       <c r="A48" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>34</v>
@@ -1331,7 +1378,7 @@
         <v>9</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="43.2">
@@ -1345,7 +1392,7 @@
         <v>37</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="28.8">
@@ -1359,7 +1406,7 @@
         <v>9</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="57.6">
@@ -1370,25 +1417,25 @@
         <v>21</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="18">
       <c r="A53" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="23.4">
       <c r="A59" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="28.8">
@@ -1407,7 +1454,7 @@
     </row>
     <row r="62" spans="1:4" ht="57.6">
       <c r="A62" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>4</v>
@@ -1416,21 +1463,21 @@
         <v>5</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="129.6">
       <c r="A63" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4">
@@ -1441,7 +1488,7 @@
         <v>36</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>41</v>
@@ -1455,10 +1502,10 @@
         <v>36</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="86.4">
@@ -1472,26 +1519,26 @@
         <v>9</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="72">
       <c r="A67" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72">
       <c r="A68" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>34</v>
@@ -1500,7 +1547,7 @@
         <v>9</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="72">
@@ -1514,12 +1561,12 @@
         <v>9</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="72">
       <c r="A70" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>34</v>
@@ -1528,7 +1575,7 @@
         <v>9</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="72">
@@ -1542,7 +1589,7 @@
         <v>9</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="60" customHeight="1">
@@ -1556,12 +1603,12 @@
         <v>9</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="201.6">
       <c r="A73" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>28</v>
@@ -1570,10 +1617,10 @@
         <v>37</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="72">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="129.6">
       <c r="A74" s="2" t="s">
         <v>48</v>
       </c>
@@ -1584,469 +1631,480 @@
         <v>37</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="57.6">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="72">
       <c r="A75" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="57.6">
+      <c r="A76" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B76" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C75" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="18">
-      <c r="A78" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4">
-      <c r="A80" s="4" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="23.4">
-      <c r="A84" s="3" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" ht="28.8">
-      <c r="A86" s="1" t="s">
+      <c r="C76" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="18">
+      <c r="A79" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
+      <c r="A81" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
+      <c r="A83" s="9" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="61.8" customHeight="1">
+      <c r="A84" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B84" s="10"/>
+      <c r="C84" s="10"/>
+      <c r="D84" s="10"/>
+    </row>
+    <row r="86" spans="1:4" ht="79.2" customHeight="1">
+      <c r="A86" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B86" s="10"/>
+      <c r="C86" s="10"/>
+      <c r="D86" s="10"/>
+    </row>
+    <row r="90" spans="1:4" ht="23.4">
+      <c r="A90" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="28.8">
+      <c r="A92" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="B92" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C86" s="1" t="s">
+      <c r="C92" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D86" s="1" t="s">
+      <c r="D92" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="57.6">
-      <c r="A87" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B87" s="2" t="s">
+    <row r="93" spans="1:4" ht="57.6">
+      <c r="A93" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B93" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="C93" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D87" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" ht="72">
-      <c r="A88" s="2" t="s">
+      <c r="D93" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="72">
+      <c r="A94" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="B94" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C88" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" ht="86.4">
-      <c r="A89" s="2" t="s">
+      <c r="C94" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="86.4">
+      <c r="A95" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B95" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="C95" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="86.4">
+      <c r="A96" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" ht="57.6">
+      <c r="A97" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" ht="72">
+      <c r="A98" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" ht="72">
+      <c r="A99" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="18">
+      <c r="A101" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4">
+      <c r="A103" s="4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" ht="23.4">
+      <c r="A107" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="28.8">
+      <c r="A109" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="57.6">
+      <c r="A110" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" ht="100.8">
+      <c r="A111" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" ht="86.4">
+      <c r="A112" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" ht="100.8">
+      <c r="A113" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="18">
+      <c r="A115" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4">
+      <c r="A117" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D89" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" ht="86.4">
-      <c r="A90" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B90" s="2" t="s">
+    </row>
+    <row r="121" spans="1:4" ht="23.4">
+      <c r="A121" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" ht="28.8">
+      <c r="A123" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" ht="57.6">
+      <c r="A124" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" ht="86.4">
+      <c r="A125" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B125" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="C125" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="D90" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="57.6">
-      <c r="A91" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B91" s="2" t="s">
+      <c r="D125" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" ht="28.8">
+      <c r="A126" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B126" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C91" s="2" t="s">
+      <c r="C126" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D91" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" ht="72">
-      <c r="A92" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B92" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D92" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" ht="72">
-      <c r="A93" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B93" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" ht="18">
-      <c r="A95" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4">
-      <c r="A97" s="4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" ht="23.4">
-      <c r="A101" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" ht="28.8">
-      <c r="A103" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B103" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C103" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D103" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" ht="57.6">
-      <c r="A104" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="B104" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C104" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" ht="100.8">
-      <c r="A105" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B105" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C105" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D105" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" ht="86.4">
-      <c r="A106" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B106" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" ht="100.8">
-      <c r="A107" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" ht="18">
-      <c r="A109" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4">
-      <c r="A111" s="4" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" ht="23.4">
-      <c r="A115" s="3" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" ht="28.8">
-      <c r="A117" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B117" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C117" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D117" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" ht="57.6">
-      <c r="A118" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B118" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C118" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" ht="86.4">
-      <c r="A119" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B119" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C119" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" ht="28.8">
-      <c r="A120" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B120" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C120" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D120" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" ht="57.6">
-      <c r="A121" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="B121" s="2" t="s">
+      <c r="D126" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" ht="57.6">
+      <c r="A127" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B127" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C121" s="2" t="s">
+      <c r="C127" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D121" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" ht="57.6">
-      <c r="A122" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B122" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C122" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D122" s="2" t="s">
+      <c r="D127" s="2" t="s">
         <v>117</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" ht="43.2" customHeight="1">
-      <c r="A125" s="5" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" ht="28.8">
-      <c r="A127" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B127" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C127" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="D127" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="57.6">
       <c r="A128" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" ht="43.2" customHeight="1">
+      <c r="A131" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" ht="28.8">
+      <c r="A133" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C133" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B128" s="2" t="s">
+      <c r="D133" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" ht="57.6">
+      <c r="A134" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="C128" s="2" t="s">
+      <c r="B134" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="D128" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" ht="115.2">
-      <c r="A129" s="2" t="s">
+      <c r="C134" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" ht="115.2">
+      <c r="A135" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B129" s="2" t="s">
+      <c r="B135" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C129" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="D129" s="2" t="s">
+      <c r="C135" s="2" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="130" spans="1:4" ht="187.2">
-      <c r="A130" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B130" s="2" t="s">
+      <c r="D135" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" ht="187.2">
+      <c r="A136" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B136" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C130" s="2" t="s">
+      <c r="C136" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D130" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" ht="57.6">
-      <c r="A131" s="2" t="s">
+      <c r="D136" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" ht="57.6">
+      <c r="A137" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B131" s="2" t="s">
+      <c r="B137" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C131" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D131" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" ht="57.6">
-      <c r="A132" s="2" t="s">
+      <c r="C137" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" ht="57.6">
+      <c r="A138" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B132" s="2" t="s">
+      <c r="B138" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C132" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D132" s="2" t="s">
+      <c r="C138" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D138" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="14.4" customHeight="1"/>
-    <row r="134" spans="1:4" ht="28.8" customHeight="1">
-      <c r="A134" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" ht="40.200000000000003" customHeight="1">
-      <c r="A135" s="8"/>
-    </row>
-    <row r="136" spans="1:4" ht="27" customHeight="1">
-      <c r="A136" s="4" t="s">
+    <row r="139" spans="1:4" ht="14.4" customHeight="1"/>
+    <row r="140" spans="1:4" ht="28.8" customHeight="1">
+      <c r="A140" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="139" spans="1:4" ht="31.2">
-      <c r="A139" s="7" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" ht="18">
-      <c r="A141" s="5" t="s">
+    <row r="141" spans="1:4" ht="40.200000000000003" customHeight="1">
+      <c r="A141" s="8"/>
+    </row>
+    <row r="142" spans="1:4" ht="27" customHeight="1">
+      <c r="A142" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" ht="31.2">
+      <c r="A145" s="7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="142" spans="1:4">
-      <c r="A142" s="6"/>
-    </row>
-    <row r="143" spans="1:4">
-      <c r="A143" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4">
-      <c r="A144" s="6"/>
-    </row>
-    <row r="145" spans="1:1">
-      <c r="A145" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="146" spans="1:1">
-      <c r="A146" s="6"/>
-    </row>
-    <row r="147" spans="1:1">
-      <c r="A147" s="6" t="s">
-        <v>72</v>
+    <row r="147" spans="1:1" ht="18">
+      <c r="A147" s="5" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="148" spans="1:1">
@@ -2054,12 +2112,15 @@
     </row>
     <row r="149" spans="1:1">
       <c r="A149" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150" s="6"/>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151" s="6" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="151" spans="1:1" ht="18">
-      <c r="A151" s="5" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="152" spans="1:1">
@@ -2078,22 +2139,25 @@
         <v>60</v>
       </c>
     </row>
-    <row r="157" spans="1:1" ht="18">
-      <c r="A157" s="5" t="s">
+    <row r="156" spans="1:1">
+      <c r="A156" s="6"/>
+    </row>
+    <row r="157" spans="1:1">
+      <c r="A157" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" ht="18">
+      <c r="A159" s="5" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="158" spans="1:1">
-      <c r="A158" s="6"/>
-    </row>
-    <row r="159" spans="1:1">
-      <c r="A159" s="6" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="161" spans="1:1" ht="18">
-      <c r="A161" s="5" t="s">
-        <v>43</v>
+    <row r="160" spans="1:1">
+      <c r="A160" s="6"/>
+    </row>
+    <row r="161" spans="1:1">
+      <c r="A161" s="6" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="162" spans="1:1">
@@ -2101,10 +2165,41 @@
     </row>
     <row r="163" spans="1:1">
       <c r="A163" s="6" t="s">
-        <v>74</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" ht="18">
+      <c r="A165" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1">
+      <c r="A166" s="6"/>
+    </row>
+    <row r="167" spans="1:1">
+      <c r="A167" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" ht="18">
+      <c r="A169" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1">
+      <c r="A170" s="6"/>
+    </row>
+    <row r="171" spans="1:1">
+      <c r="A171" s="6" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A84:D84"/>
+    <mergeCell ref="A86:D86"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>